<commit_message>
feat: publish saas-magnet-cold-email-sequences (add Creative Liquidity Gap sequence)
</commit_message>
<xml_diff>
--- a/saas-magnet-cold-email-sequences/adpros_cold_email_sequences.xlsx
+++ b/saas-magnet-cold-email-sequences/adpros_cold_email_sequences.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ad Diversity Audit" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Creator Spy" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flagship Audit" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creative Liquidity Gap" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -555,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -742,27 +743,49 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
+          <t>Creative Liquidity Gap</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Format coverage analysis of their live library: static/video/carousel split, angles trapped in one format, auctions they’re locked out of</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Mechanism insight. Meta-native "creative liquidity" language, zero access needed.</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Library-based — no account access friction. Educates while it sells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
           <t>Flagship Audit</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>The 100-page competitor creative strategy audit — all magnets combined + 90-day attack plan</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Audacity. "This will sound like a lot" + downgrade close (3-page mini).</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Reserve for highest-value targets and leadership personas.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>LAUNCH PLAN: Start with Competitor Ad Spy vs. Creative Scorecard head-to-head (rivalry vs. vanity) — let reply data pick the winning psychological angle before rolling out the rest. All merge fields must be populated with real pipeline data; the specificity is the mechanism.</t>
         </is>
@@ -771,9 +794,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2133,4 +2156,198 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MAGNET — CREATIVE LIQUIDITY GAP ANALYSIS (format coverage across their live ad library)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Angle: The mechanism angle: Meta’s delivery system needs a liquid mix of formats (static / video / carousel) per angle to enter every auction. We measure their format gap from the public ads library — no account access needed — and show the auctions they’re locked out of.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>OPTIONAL P.S. (decide per sequence whether to add): "P.S. Reply and I’ll also show you how to talk to any brand’s ads library inside Claude or Slack — takes 10 minutes to set up and it’s free."</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL 1 — THE OFFER  (Day 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>{{brand}} is locked out of auctions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="238" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Hi {{first_name}},
+Meta’s delivery system works like a liquidity market: to find the cheapest conversion for each person, it needs every angle available in every format — static, video, carousel. If an angle only exists as video, you never enter the auctions where a static or carousel would have won. Meta calls this creative liquidity.
+We analyzed {{brand}}’s live ad library: {{X}} active ads, {{static_pct}} static / {{video_pct}} video / {{carousel_pct}} carousel — and {{gap_count}} of your angles exist in only ONE format.
+That’s {{gap_count}} sets of auctions you’re structurally locked out of, every day.
+Want the full liquidity gap analysis? It maps every angle, every missing format, and what to produce first. Just reply “liquidity.”
+Nehal
+Founder, Ad Pros</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>All variables pull from public ads library — zero access friction. {{gap_count}} is the gut-punch number. Format percentages prove real analysis happened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL 2 — THE MECHANISM  (Day 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>why single-format angles cost more</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="280" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>{{first_name}},
+Quick context on why the format gap matters more than most teams realize — three compounding effects:
+1. Auction lockout — someone who only watches Reels never sees your feed-only angle. That demand goes to a competitor by default.
+2. Self-competition — when the same angle is split across many near-duplicate ads instead of one liquid set, your ads bid against each other, inflating your own CPMs.
+3. Slower learning — the system needs roughly 50 conversions a week per ad set to stabilize. Fragmented formats starve every set of data; consolidated liquid sets exit learning faster and deliver cheaper.
+The analysis shows exactly where {{brand}} sits on all three. Reply “liquidity” and I’ll send it over.
+Nehal
+Founder, Ad Pros</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>The only email in the playbook with a numbered list — the mechanism has three genuinely distinct parts and teaching them builds authority. Keeps the library-based promise: analysis is format coverage; mechanism education covers the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL 3 — BREAKUP + GIVE  (Day 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>your biggest liquidity gap (free)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="182" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>{{first_name}} — last note, and here’s the headline for free:
+Your “{{top_angle}}” angle — one of your longest-running — exists only as {{existing_format}}. No {{missing_format_1}}, no {{missing_format_2}}. Your best-proven message is invisible to everyone whose feed behavior favors those formats.
+That’s one angle. The full analysis covers all of them, ranked by how much reach each gap is costing you.
+Reply “liquidity” if you want it — or just go make those two assets. Either way you win.
+Nehal
+Founder, Ad Pros</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>“Either way you win” is the confidence close — giving away actionable advice signals abundance. {{top_angle}} must be their genuinely longest-running ad’s angle for the gift to land.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>